<commit_message>
Início da organização da licença de uso.
</commit_message>
<xml_diff>
--- a/dados/microrregioes_final.xlsx
+++ b/dados/microrregioes_final.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\desenvolvimentos\apps\gd_impacta_mg\dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Documents\dev_2026\gd_impacta_mg\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4997E5DB-7675-4B31-8CD3-C6564C176CAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AFFE15B-18C6-4E1D-811F-49E85A452EEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{C5D685B8-32F5-4BB9-B9E4-7E8B786E1705}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{C5D685B8-32F5-4BB9-B9E4-7E8B786E1705}"/>
   </bookViews>
   <sheets>
     <sheet name="Agregados - Micro" sheetId="1" r:id="rId1"/>
     <sheet name="Produção - Micro" sheetId="2" r:id="rId2"/>
     <sheet name="Investimento - Micro" sheetId="4" r:id="rId3"/>
+    <sheet name="ICMS - Micro" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="85">
   <si>
     <t>cenario</t>
   </si>
@@ -668,12 +669,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E8A1431-C631-45DF-91E4-F1D9A56B9AAA}">
   <dimension ref="A1:BP17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -879,7 +880,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>75</v>
       </c>
@@ -1085,7 +1086,7 @@
         <v>10.641999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>75</v>
       </c>
@@ -1291,7 +1292,7 @@
         <v>5.6859999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -1497,7 +1498,7 @@
         <v>3.0870000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>75</v>
       </c>
@@ -1703,7 +1704,7 @@
         <v>3.9689999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>75</v>
       </c>
@@ -1909,7 +1910,7 @@
         <v>3.7240000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>75</v>
       </c>
@@ -2115,7 +2116,7 @@
         <v>1.9339999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>75</v>
       </c>
@@ -2321,7 +2322,7 @@
         <v>6.343</v>
       </c>
     </row>
-    <row r="9" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>75</v>
       </c>
@@ -2527,7 +2528,7 @@
         <v>-3.25</v>
       </c>
     </row>
-    <row r="10" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>76</v>
       </c>
@@ -2733,7 +2734,7 @@
         <v>10.973000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>76</v>
       </c>
@@ -2939,7 +2940,7 @@
         <v>5.8460000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>76</v>
       </c>
@@ -3145,7 +3146,7 @@
         <v>3.3730000000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>76</v>
       </c>
@@ -3351,7 +3352,7 @@
         <v>3.9009999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>76</v>
       </c>
@@ -3557,7 +3558,7 @@
         <v>3.7789999999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>76</v>
       </c>
@@ -3763,7 +3764,7 @@
         <v>1.9179999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>76</v>
       </c>
@@ -3969,7 +3970,7 @@
         <v>6.6950000000000003</v>
       </c>
     </row>
-    <row r="17" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>76</v>
       </c>
@@ -4183,13 +4184,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F663516-9BA9-4400-A0A6-8CB898693602}">
   <dimension ref="A1:BP13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4395,7 +4396,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -4601,7 +4602,7 @@
         <v>5.6479999999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -4807,7 +4808,7 @@
         <v>6.7389999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -5013,7 +5014,7 @@
         <v>6.9560000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -5219,7 +5220,7 @@
         <v>1.9830000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -5425,7 +5426,7 @@
         <v>7.2389999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>78</v>
       </c>
@@ -5631,7 +5632,7 @@
         <v>4.8230000000000004</v>
       </c>
     </row>
-    <row r="8" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -5837,7 +5838,7 @@
         <v>5.8550000000000004</v>
       </c>
     </row>
-    <row r="9" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>76</v>
       </c>
@@ -6043,7 +6044,7 @@
         <v>7.609</v>
       </c>
     </row>
-    <row r="10" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>76</v>
       </c>
@@ -6249,7 +6250,7 @@
         <v>7.32</v>
       </c>
     </row>
-    <row r="11" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>76</v>
       </c>
@@ -6455,7 +6456,7 @@
         <v>1.9179999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>76</v>
       </c>
@@ -6661,7 +6662,7 @@
         <v>7.6959999999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>76</v>
       </c>
@@ -6875,13 +6876,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA292EC3-8AF3-4031-96CF-4119299986AF}">
   <dimension ref="A1:BP13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7087,7 +7088,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -7293,7 +7294,7 @@
         <v>7.1849999999999996</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -7499,7 +7500,7 @@
         <v>8.3870000000000005</v>
       </c>
     </row>
-    <row r="4" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -7705,7 +7706,7 @@
         <v>9.3360000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -7911,7 +7912,7 @@
         <v>4.3220000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -8117,7 +8118,7 @@
         <v>9.202</v>
       </c>
     </row>
-    <row r="7" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>78</v>
       </c>
@@ -8323,7 +8324,7 @@
         <v>6.9210000000000003</v>
       </c>
     </row>
-    <row r="8" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -8529,7 +8530,7 @@
         <v>7.4530000000000003</v>
       </c>
     </row>
-    <row r="9" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>76</v>
       </c>
@@ -8735,7 +8736,7 @@
         <v>9.33</v>
       </c>
     </row>
-    <row r="10" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>76</v>
       </c>
@@ -8941,7 +8942,7 @@
         <v>9.7989999999999995</v>
       </c>
     </row>
-    <row r="11" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>76</v>
       </c>
@@ -9147,7 +9148,7 @@
         <v>4.3470000000000004</v>
       </c>
     </row>
-    <row r="12" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>76</v>
       </c>
@@ -9353,7 +9354,7 @@
         <v>9.7430000000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:68" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>76</v>
       </c>
@@ -9557,6 +9558,2698 @@
       </c>
       <c r="BP13">
         <v>7.2690000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A98E2AA3-1555-4AFC-99D6-8CB391DD4AE6}">
+  <dimension ref="A1:BP13"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" t="s">
+        <v>21</v>
+      </c>
+      <c r="P1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>23</v>
+      </c>
+      <c r="R1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U1" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" t="s">
+        <v>28</v>
+      </c>
+      <c r="W1" t="s">
+        <v>29</v>
+      </c>
+      <c r="X1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>64</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>65</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>66</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>71</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2">
+        <v>9160006.1507273652</v>
+      </c>
+      <c r="D2">
+        <v>44163670.925292552</v>
+      </c>
+      <c r="E2">
+        <v>11135930.718462853</v>
+      </c>
+      <c r="F2">
+        <v>7366279.3006459475</v>
+      </c>
+      <c r="G2">
+        <v>7762681.4649032801</v>
+      </c>
+      <c r="H2">
+        <v>63957841.233583502</v>
+      </c>
+      <c r="I2">
+        <v>13924954.295081425</v>
+      </c>
+      <c r="J2">
+        <v>57141449.506359123</v>
+      </c>
+      <c r="K2">
+        <v>9256338.6510273814</v>
+      </c>
+      <c r="L2">
+        <v>34293879.348691545</v>
+      </c>
+      <c r="M2">
+        <v>11187578.589499146</v>
+      </c>
+      <c r="N2">
+        <v>18020770.767551478</v>
+      </c>
+      <c r="O2">
+        <v>27459041.439801432</v>
+      </c>
+      <c r="P2">
+        <v>13481051.786436357</v>
+      </c>
+      <c r="Q2">
+        <v>3748455.7966076205</v>
+      </c>
+      <c r="R2">
+        <v>11637734.790623032</v>
+      </c>
+      <c r="S2">
+        <v>17535238.594494566</v>
+      </c>
+      <c r="T2">
+        <v>7046510.854199213</v>
+      </c>
+      <c r="U2">
+        <v>42745987.901131503</v>
+      </c>
+      <c r="V2">
+        <v>20734820.457007863</v>
+      </c>
+      <c r="W2">
+        <v>31801972.781569</v>
+      </c>
+      <c r="X2">
+        <v>27623494.972243797</v>
+      </c>
+      <c r="Y2">
+        <v>1387772.1847095639</v>
+      </c>
+      <c r="Z2">
+        <v>8214312.0756365051</v>
+      </c>
+      <c r="AA2">
+        <v>10912182.958856964</v>
+      </c>
+      <c r="AB2">
+        <v>12860668.024537282</v>
+      </c>
+      <c r="AC2">
+        <v>10890889.997778557</v>
+      </c>
+      <c r="AD2">
+        <v>12444290.952087337</v>
+      </c>
+      <c r="AE2">
+        <v>21255552.898475274</v>
+      </c>
+      <c r="AF2">
+        <v>30105173.041448608</v>
+      </c>
+      <c r="AG2">
+        <v>32430629.608825199</v>
+      </c>
+      <c r="AH2">
+        <v>19408596.069194701</v>
+      </c>
+      <c r="AI2">
+        <v>12712447.056432368</v>
+      </c>
+      <c r="AJ2">
+        <v>32969942.818386029</v>
+      </c>
+      <c r="AK2">
+        <v>7670595.4781576404</v>
+      </c>
+      <c r="AL2">
+        <v>24452289.61096577</v>
+      </c>
+      <c r="AM2">
+        <v>30901122.033610437</v>
+      </c>
+      <c r="AN2">
+        <v>11553371.341334401</v>
+      </c>
+      <c r="AO2">
+        <v>23783023.135009922</v>
+      </c>
+      <c r="AP2">
+        <v>3236821.1741261552</v>
+      </c>
+      <c r="AQ2">
+        <v>20800558.915267602</v>
+      </c>
+      <c r="AR2">
+        <v>59654698.380956128</v>
+      </c>
+      <c r="AS2">
+        <v>44513810.546184607</v>
+      </c>
+      <c r="AT2">
+        <v>46030132.286730312</v>
+      </c>
+      <c r="AU2">
+        <v>52055717.982130811</v>
+      </c>
+      <c r="AV2">
+        <v>9644549.2900089156</v>
+      </c>
+      <c r="AW2">
+        <v>4197543.976781711</v>
+      </c>
+      <c r="AX2">
+        <v>17713696.438848529</v>
+      </c>
+      <c r="AY2">
+        <v>8456881.7412736304</v>
+      </c>
+      <c r="AZ2">
+        <v>23595247.833443455</v>
+      </c>
+      <c r="BA2">
+        <v>20507476.769227393</v>
+      </c>
+      <c r="BB2">
+        <v>19166610.931001052</v>
+      </c>
+      <c r="BC2">
+        <v>9296117.0755968746</v>
+      </c>
+      <c r="BD2">
+        <v>12630279.754118428</v>
+      </c>
+      <c r="BE2">
+        <v>21441503.459843494</v>
+      </c>
+      <c r="BF2">
+        <v>30299379.315465834</v>
+      </c>
+      <c r="BG2">
+        <v>32735654.470936377</v>
+      </c>
+      <c r="BH2">
+        <v>41235430.130230203</v>
+      </c>
+      <c r="BI2">
+        <v>25834305.637690727</v>
+      </c>
+      <c r="BJ2">
+        <v>20530115.188705876</v>
+      </c>
+      <c r="BK2">
+        <v>23117974.296525694</v>
+      </c>
+      <c r="BL2">
+        <v>64168799.117908157</v>
+      </c>
+      <c r="BM2">
+        <v>74189819.575156748</v>
+      </c>
+      <c r="BN2">
+        <v>62543184.462895237</v>
+      </c>
+      <c r="BO2">
+        <v>69050568.110917807</v>
+      </c>
+      <c r="BP2">
+        <v>30060079.564734828</v>
+      </c>
+    </row>
+    <row r="3" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3">
+        <v>11206558.134800503</v>
+      </c>
+      <c r="D3">
+        <v>36069955.102446638</v>
+      </c>
+      <c r="E3">
+        <v>4423011.4104796741</v>
+      </c>
+      <c r="F3">
+        <v>1838491.4070472233</v>
+      </c>
+      <c r="G3">
+        <v>4917106.2667592727</v>
+      </c>
+      <c r="H3">
+        <v>139666546.25626424</v>
+      </c>
+      <c r="I3">
+        <v>18885560.36304957</v>
+      </c>
+      <c r="J3">
+        <v>4827087750.8676748</v>
+      </c>
+      <c r="K3">
+        <v>5918247.7213728521</v>
+      </c>
+      <c r="L3">
+        <v>22107121.899742603</v>
+      </c>
+      <c r="M3">
+        <v>8466955.1633243933</v>
+      </c>
+      <c r="N3">
+        <v>6085287.5129616279</v>
+      </c>
+      <c r="O3">
+        <v>8408957.800952727</v>
+      </c>
+      <c r="P3">
+        <v>49799632.607435532</v>
+      </c>
+      <c r="Q3">
+        <v>66541837.548304439</v>
+      </c>
+      <c r="R3">
+        <v>487281803.13359958</v>
+      </c>
+      <c r="S3">
+        <v>6303934.8240490425</v>
+      </c>
+      <c r="T3">
+        <v>4295340.6888937922</v>
+      </c>
+      <c r="U3">
+        <v>260232389.54110777</v>
+      </c>
+      <c r="V3">
+        <v>25304774.366856974</v>
+      </c>
+      <c r="W3">
+        <v>62234211.76289212</v>
+      </c>
+      <c r="X3">
+        <v>27821150.335896876</v>
+      </c>
+      <c r="Y3">
+        <v>4966867.0872999383</v>
+      </c>
+      <c r="Z3">
+        <v>7248272.048317587</v>
+      </c>
+      <c r="AA3">
+        <v>417318277.56734967</v>
+      </c>
+      <c r="AB3">
+        <v>656693450.58565235</v>
+      </c>
+      <c r="AC3">
+        <v>120838488.01242857</v>
+      </c>
+      <c r="AD3">
+        <v>28910955.283485111</v>
+      </c>
+      <c r="AE3">
+        <v>22682260.871981293</v>
+      </c>
+      <c r="AF3">
+        <v>52430299.159050047</v>
+      </c>
+      <c r="AG3">
+        <v>6629796.1754419198</v>
+      </c>
+      <c r="AH3">
+        <v>117070124.62527081</v>
+      </c>
+      <c r="AI3">
+        <v>16495981.682790481</v>
+      </c>
+      <c r="AJ3">
+        <v>58013725.159097865</v>
+      </c>
+      <c r="AK3">
+        <v>1556510.1543323125</v>
+      </c>
+      <c r="AL3">
+        <v>39033619.055373736</v>
+      </c>
+      <c r="AM3">
+        <v>47789527.602822781</v>
+      </c>
+      <c r="AN3">
+        <v>6716215.67051691</v>
+      </c>
+      <c r="AO3">
+        <v>29181333.198271468</v>
+      </c>
+      <c r="AP3">
+        <v>752149915.01768374</v>
+      </c>
+      <c r="AQ3">
+        <v>21971889.564977776</v>
+      </c>
+      <c r="AR3">
+        <v>123241898.04355483</v>
+      </c>
+      <c r="AS3">
+        <v>58313515.692903034</v>
+      </c>
+      <c r="AT3">
+        <v>20774702.081062529</v>
+      </c>
+      <c r="AU3">
+        <v>18972370.254469432</v>
+      </c>
+      <c r="AV3">
+        <v>1130202.1412240921</v>
+      </c>
+      <c r="AW3">
+        <v>3548224.7518607033</v>
+      </c>
+      <c r="AX3">
+        <v>16291488.691442901</v>
+      </c>
+      <c r="AY3">
+        <v>5208307.7903416939</v>
+      </c>
+      <c r="AZ3">
+        <v>116302502.96219037</v>
+      </c>
+      <c r="BA3">
+        <v>12083582.978606023</v>
+      </c>
+      <c r="BB3">
+        <v>101002702.14672071</v>
+      </c>
+      <c r="BC3">
+        <v>11140475.651774589</v>
+      </c>
+      <c r="BD3">
+        <v>18807174.255482066</v>
+      </c>
+      <c r="BE3">
+        <v>55339615.188878462</v>
+      </c>
+      <c r="BF3">
+        <v>14912078.899907174</v>
+      </c>
+      <c r="BG3">
+        <v>50695947.593657367</v>
+      </c>
+      <c r="BH3">
+        <v>78984175.077279031</v>
+      </c>
+      <c r="BI3">
+        <v>8733375.4923835378</v>
+      </c>
+      <c r="BJ3">
+        <v>37298661.006025977</v>
+      </c>
+      <c r="BK3">
+        <v>42115041.891475841</v>
+      </c>
+      <c r="BL3">
+        <v>141066636.66385332</v>
+      </c>
+      <c r="BM3">
+        <v>276505197.40778714</v>
+      </c>
+      <c r="BN3">
+        <v>21546477.36362014</v>
+      </c>
+      <c r="BO3">
+        <v>58767863.652826995</v>
+      </c>
+      <c r="BP3">
+        <v>8617322.5678500962</v>
+      </c>
+    </row>
+    <row r="4" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4">
+        <v>112144458.48794663</v>
+      </c>
+      <c r="D4">
+        <v>802159789.62120545</v>
+      </c>
+      <c r="E4">
+        <v>134305463.66715044</v>
+      </c>
+      <c r="F4">
+        <v>11186790.218775338</v>
+      </c>
+      <c r="G4">
+        <v>99868934.004311204</v>
+      </c>
+      <c r="H4">
+        <v>3487230956.7410121</v>
+      </c>
+      <c r="I4">
+        <v>774880028.31889486</v>
+      </c>
+      <c r="J4">
+        <v>21017524380.640312</v>
+      </c>
+      <c r="K4">
+        <v>1964274927.8112934</v>
+      </c>
+      <c r="L4">
+        <v>631629206.36952889</v>
+      </c>
+      <c r="M4">
+        <v>189488435.73542479</v>
+      </c>
+      <c r="N4">
+        <v>353440666.57396829</v>
+      </c>
+      <c r="O4">
+        <v>405876360.04839617</v>
+      </c>
+      <c r="P4">
+        <v>583734302.29940426</v>
+      </c>
+      <c r="Q4">
+        <v>204678410.83862752</v>
+      </c>
+      <c r="R4">
+        <v>5410394867.3514538</v>
+      </c>
+      <c r="S4">
+        <v>284608283.78347719</v>
+      </c>
+      <c r="T4">
+        <v>104548229.67938255</v>
+      </c>
+      <c r="U4">
+        <v>3996666180.3102422</v>
+      </c>
+      <c r="V4">
+        <v>924286338.21846366</v>
+      </c>
+      <c r="W4">
+        <v>303773577.3666628</v>
+      </c>
+      <c r="X4">
+        <v>809373726.13578796</v>
+      </c>
+      <c r="Y4">
+        <v>130433574.39832538</v>
+      </c>
+      <c r="Z4">
+        <v>236456013.49743694</v>
+      </c>
+      <c r="AA4">
+        <v>7552394062.3097935</v>
+      </c>
+      <c r="AB4">
+        <v>5365759473.8486891</v>
+      </c>
+      <c r="AC4">
+        <v>1339841403.249325</v>
+      </c>
+      <c r="AD4">
+        <v>261231922.41310084</v>
+      </c>
+      <c r="AE4">
+        <v>735554786.14202416</v>
+      </c>
+      <c r="AF4">
+        <v>372225095.67994273</v>
+      </c>
+      <c r="AG4">
+        <v>375450085.4638685</v>
+      </c>
+      <c r="AH4">
+        <v>5971276497.3362713</v>
+      </c>
+      <c r="AI4">
+        <v>244802213.5580042</v>
+      </c>
+      <c r="AJ4">
+        <v>971233423.89643455</v>
+      </c>
+      <c r="AK4">
+        <v>48892084.805472061</v>
+      </c>
+      <c r="AL4">
+        <v>1403962710.0201004</v>
+      </c>
+      <c r="AM4">
+        <v>416207213.66316414</v>
+      </c>
+      <c r="AN4">
+        <v>53723331.742295593</v>
+      </c>
+      <c r="AO4">
+        <v>326220137.03088129</v>
+      </c>
+      <c r="AP4">
+        <v>4798781913.7658243</v>
+      </c>
+      <c r="AQ4">
+        <v>877689922.6892463</v>
+      </c>
+      <c r="AR4">
+        <v>709073042.10025883</v>
+      </c>
+      <c r="AS4">
+        <v>1174916758.5469759</v>
+      </c>
+      <c r="AT4">
+        <v>866197927.12217367</v>
+      </c>
+      <c r="AU4">
+        <v>594288935.89888036</v>
+      </c>
+      <c r="AV4">
+        <v>22163364.55746847</v>
+      </c>
+      <c r="AW4">
+        <v>91048503.656478062</v>
+      </c>
+      <c r="AX4">
+        <v>1892044193.117547</v>
+      </c>
+      <c r="AY4">
+        <v>269865242.24600244</v>
+      </c>
+      <c r="AZ4">
+        <v>2293720533.0401125</v>
+      </c>
+      <c r="BA4">
+        <v>202270449.47124013</v>
+      </c>
+      <c r="BB4">
+        <v>1547779423.2463441</v>
+      </c>
+      <c r="BC4">
+        <v>536953127.48635328</v>
+      </c>
+      <c r="BD4">
+        <v>-87576106.588372469</v>
+      </c>
+      <c r="BE4">
+        <v>648294373.91517305</v>
+      </c>
+      <c r="BF4">
+        <v>420733785.43630672</v>
+      </c>
+      <c r="BG4">
+        <v>788736504.64897382</v>
+      </c>
+      <c r="BH4">
+        <v>2833108015.7236733</v>
+      </c>
+      <c r="BI4">
+        <v>373064957.20187932</v>
+      </c>
+      <c r="BJ4">
+        <v>7393851613.9847546</v>
+      </c>
+      <c r="BK4">
+        <v>1014777261.8426535</v>
+      </c>
+      <c r="BL4">
+        <v>3552463516.6489148</v>
+      </c>
+      <c r="BM4">
+        <v>6204707948.7792463</v>
+      </c>
+      <c r="BN4">
+        <v>469771642.75407869</v>
+      </c>
+      <c r="BO4">
+        <v>1475400514.1730111</v>
+      </c>
+      <c r="BP4">
+        <v>238252099.53451517</v>
+      </c>
+    </row>
+    <row r="5" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5">
+        <v>41283003.960488625</v>
+      </c>
+      <c r="D5">
+        <v>51914801.473237738</v>
+      </c>
+      <c r="E5">
+        <v>40185378.354062594</v>
+      </c>
+      <c r="F5">
+        <v>28763010.26732754</v>
+      </c>
+      <c r="G5">
+        <v>31140302.277500764</v>
+      </c>
+      <c r="H5">
+        <v>149840137.36130917</v>
+      </c>
+      <c r="I5">
+        <v>51758552.416858412</v>
+      </c>
+      <c r="J5">
+        <v>1745153515.9367554</v>
+      </c>
+      <c r="K5">
+        <v>38303174.203421988</v>
+      </c>
+      <c r="L5">
+        <v>113959119.76199068</v>
+      </c>
+      <c r="M5">
+        <v>59976784.811547831</v>
+      </c>
+      <c r="N5">
+        <v>42874740.867014579</v>
+      </c>
+      <c r="O5">
+        <v>33164221.14965342</v>
+      </c>
+      <c r="P5">
+        <v>64757670.397132695</v>
+      </c>
+      <c r="Q5">
+        <v>14307470.549057685</v>
+      </c>
+      <c r="R5">
+        <v>98729913.013641655</v>
+      </c>
+      <c r="S5">
+        <v>115092023.69113575</v>
+      </c>
+      <c r="T5">
+        <v>21615746.884205393</v>
+      </c>
+      <c r="U5">
+        <v>330745288.8472448</v>
+      </c>
+      <c r="V5">
+        <v>145470164.48881674</v>
+      </c>
+      <c r="W5">
+        <v>157798640.90209529</v>
+      </c>
+      <c r="X5">
+        <v>97040953.468592793</v>
+      </c>
+      <c r="Y5">
+        <v>3740007.9878666122</v>
+      </c>
+      <c r="Z5">
+        <v>25402949.047406163</v>
+      </c>
+      <c r="AA5">
+        <v>251117046.62428954</v>
+      </c>
+      <c r="AB5">
+        <v>239482509.47789407</v>
+      </c>
+      <c r="AC5">
+        <v>45722365.722468317</v>
+      </c>
+      <c r="AD5">
+        <v>51939811.002617367</v>
+      </c>
+      <c r="AE5">
+        <v>64458960.052700125</v>
+      </c>
+      <c r="AF5">
+        <v>40210567.56015455</v>
+      </c>
+      <c r="AG5">
+        <v>36311620.365203969</v>
+      </c>
+      <c r="AH5">
+        <v>93968424.529148981</v>
+      </c>
+      <c r="AI5">
+        <v>97280860.849624634</v>
+      </c>
+      <c r="AJ5">
+        <v>60663415.782126851</v>
+      </c>
+      <c r="AK5">
+        <v>8419862.7117004525</v>
+      </c>
+      <c r="AL5">
+        <v>484451734.9277178</v>
+      </c>
+      <c r="AM5">
+        <v>85826091.953661457</v>
+      </c>
+      <c r="AN5">
+        <v>13328194.203977099</v>
+      </c>
+      <c r="AO5">
+        <v>31183917.986767218</v>
+      </c>
+      <c r="AP5">
+        <v>137781390.55662578</v>
+      </c>
+      <c r="AQ5">
+        <v>46132236.280852698</v>
+      </c>
+      <c r="AR5">
+        <v>344861441.9853605</v>
+      </c>
+      <c r="AS5">
+        <v>99609173.796946242</v>
+      </c>
+      <c r="AT5">
+        <v>160714093.71025056</v>
+      </c>
+      <c r="AU5">
+        <v>130046236.09974515</v>
+      </c>
+      <c r="AV5">
+        <v>2709265.6046089488</v>
+      </c>
+      <c r="AW5">
+        <v>8584397.7094201948</v>
+      </c>
+      <c r="AX5">
+        <v>137941779.28033847</v>
+      </c>
+      <c r="AY5">
+        <v>131410894.81172942</v>
+      </c>
+      <c r="AZ5">
+        <v>156844453.53397253</v>
+      </c>
+      <c r="BA5">
+        <v>50970571.299184255</v>
+      </c>
+      <c r="BB5">
+        <v>86383977.698840156</v>
+      </c>
+      <c r="BC5">
+        <v>121709226.50494757</v>
+      </c>
+      <c r="BD5">
+        <v>61757010.473893344</v>
+      </c>
+      <c r="BE5">
+        <v>16359416.767499043</v>
+      </c>
+      <c r="BF5">
+        <v>75670744.172793031</v>
+      </c>
+      <c r="BG5">
+        <v>121981624.91817755</v>
+      </c>
+      <c r="BH5">
+        <v>440189916.85753083</v>
+      </c>
+      <c r="BI5">
+        <v>86659331.143866464</v>
+      </c>
+      <c r="BJ5">
+        <v>48063825.361234181</v>
+      </c>
+      <c r="BK5">
+        <v>94102335.664742664</v>
+      </c>
+      <c r="BL5">
+        <v>118884899.46104324</v>
+      </c>
+      <c r="BM5">
+        <v>396066975.14533496</v>
+      </c>
+      <c r="BN5">
+        <v>42283069.34907496</v>
+      </c>
+      <c r="BO5">
+        <v>215395563.71358275</v>
+      </c>
+      <c r="BP5">
+        <v>30966489.797677282</v>
+      </c>
+    </row>
+    <row r="6" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6">
+        <v>335993663.99932498</v>
+      </c>
+      <c r="D6">
+        <v>1154866377.7792056</v>
+      </c>
+      <c r="E6">
+        <v>322580484.4854582</v>
+      </c>
+      <c r="F6">
+        <v>115299957.17355426</v>
+      </c>
+      <c r="G6">
+        <v>180669082.77093425</v>
+      </c>
+      <c r="H6">
+        <v>1350056956.9727032</v>
+      </c>
+      <c r="I6">
+        <v>662320353.32645321</v>
+      </c>
+      <c r="J6">
+        <v>27074272351.443882</v>
+      </c>
+      <c r="K6">
+        <v>252674379.75995538</v>
+      </c>
+      <c r="L6">
+        <v>1086137911.900954</v>
+      </c>
+      <c r="M6">
+        <v>371868189.37859505</v>
+      </c>
+      <c r="N6">
+        <v>516818109.82208765</v>
+      </c>
+      <c r="O6">
+        <v>830395344.33662128</v>
+      </c>
+      <c r="P6">
+        <v>807812208.01235986</v>
+      </c>
+      <c r="Q6">
+        <v>152501531.73399457</v>
+      </c>
+      <c r="R6">
+        <v>1094250924.8371778</v>
+      </c>
+      <c r="S6">
+        <v>612823071.48615336</v>
+      </c>
+      <c r="T6">
+        <v>305456129.11885315</v>
+      </c>
+      <c r="U6">
+        <v>3382352986.8827209</v>
+      </c>
+      <c r="V6">
+        <v>766022622.75296187</v>
+      </c>
+      <c r="W6">
+        <v>1258624622.9951444</v>
+      </c>
+      <c r="X6">
+        <v>2079321784.5928781</v>
+      </c>
+      <c r="Y6">
+        <v>43943470.471107736</v>
+      </c>
+      <c r="Z6">
+        <v>297638190.99587148</v>
+      </c>
+      <c r="AA6">
+        <v>2764077188.5713277</v>
+      </c>
+      <c r="AB6">
+        <v>1726689904.9714322</v>
+      </c>
+      <c r="AC6">
+        <v>264138043.11296183</v>
+      </c>
+      <c r="AD6">
+        <v>551913699.64716148</v>
+      </c>
+      <c r="AE6">
+        <v>774693488.66356981</v>
+      </c>
+      <c r="AF6">
+        <v>586008997.20540524</v>
+      </c>
+      <c r="AG6">
+        <v>793500261.56279171</v>
+      </c>
+      <c r="AH6">
+        <v>3428603279.4059758</v>
+      </c>
+      <c r="AI6">
+        <v>574875313.23883736</v>
+      </c>
+      <c r="AJ6">
+        <v>1042509181.4569609</v>
+      </c>
+      <c r="AK6">
+        <v>185102569.3355937</v>
+      </c>
+      <c r="AL6">
+        <v>2564023521.5518041</v>
+      </c>
+      <c r="AM6">
+        <v>876723083.66870904</v>
+      </c>
+      <c r="AN6">
+        <v>216202247.12864804</v>
+      </c>
+      <c r="AO6">
+        <v>464850225.68283165</v>
+      </c>
+      <c r="AP6">
+        <v>962424529.02012897</v>
+      </c>
+      <c r="AQ6">
+        <v>787339055.91887891</v>
+      </c>
+      <c r="AR6">
+        <v>816930032.12038577</v>
+      </c>
+      <c r="AS6">
+        <v>1050891356.8589214</v>
+      </c>
+      <c r="AT6">
+        <v>1535384620.9296474</v>
+      </c>
+      <c r="AU6">
+        <v>1158501902.173538</v>
+      </c>
+      <c r="AV6">
+        <v>124509055.17431433</v>
+      </c>
+      <c r="AW6">
+        <v>167464139.02351281</v>
+      </c>
+      <c r="AX6">
+        <v>745808167.77539885</v>
+      </c>
+      <c r="AY6">
+        <v>398921723.5933392</v>
+      </c>
+      <c r="AZ6">
+        <v>1916403048.7928376</v>
+      </c>
+      <c r="BA6">
+        <v>541190211.64196908</v>
+      </c>
+      <c r="BB6">
+        <v>2304497028.5949426</v>
+      </c>
+      <c r="BC6">
+        <v>673333556.02226281</v>
+      </c>
+      <c r="BD6">
+        <v>472491474.22411609</v>
+      </c>
+      <c r="BE6">
+        <v>627278983.0424701</v>
+      </c>
+      <c r="BF6">
+        <v>679711618.71122897</v>
+      </c>
+      <c r="BG6">
+        <v>1604316766.8674073</v>
+      </c>
+      <c r="BH6">
+        <v>2081947044.6423588</v>
+      </c>
+      <c r="BI6">
+        <v>836358405.0620892</v>
+      </c>
+      <c r="BJ6">
+        <v>561280426.1116451</v>
+      </c>
+      <c r="BK6">
+        <v>1036864977.7693886</v>
+      </c>
+      <c r="BL6">
+        <v>2892189417.7486405</v>
+      </c>
+      <c r="BM6">
+        <v>5709639163.3495855</v>
+      </c>
+      <c r="BN6">
+        <v>704550160.55987966</v>
+      </c>
+      <c r="BO6">
+        <v>2520397558.1555872</v>
+      </c>
+      <c r="BP6">
+        <v>652684933.83039403</v>
+      </c>
+    </row>
+    <row r="7" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7">
+        <v>4311724.1680888431</v>
+      </c>
+      <c r="D7">
+        <v>30370390.012145411</v>
+      </c>
+      <c r="E7">
+        <v>81534.267570908909</v>
+      </c>
+      <c r="F7">
+        <v>-1742950.1662494678</v>
+      </c>
+      <c r="G7">
+        <v>2284438.973808663</v>
+      </c>
+      <c r="H7">
+        <v>19103498.990562424</v>
+      </c>
+      <c r="I7">
+        <v>12601795.454406563</v>
+      </c>
+      <c r="J7">
+        <v>586646253.44250536</v>
+      </c>
+      <c r="K7">
+        <v>1118325.935867918</v>
+      </c>
+      <c r="L7">
+        <v>18864598.688847795</v>
+      </c>
+      <c r="M7">
+        <v>-1008140.9975857123</v>
+      </c>
+      <c r="N7">
+        <v>8858841.2199767269</v>
+      </c>
+      <c r="O7">
+        <v>12964228.502151851</v>
+      </c>
+      <c r="P7">
+        <v>10722997.96624309</v>
+      </c>
+      <c r="Q7">
+        <v>77999.921368476163</v>
+      </c>
+      <c r="R7">
+        <v>30565306.1565306</v>
+      </c>
+      <c r="S7">
+        <v>710213.13834772178</v>
+      </c>
+      <c r="T7">
+        <v>895689.3955652439</v>
+      </c>
+      <c r="U7">
+        <v>72426341.921685025</v>
+      </c>
+      <c r="V7">
+        <v>15598975.267023366</v>
+      </c>
+      <c r="W7">
+        <v>-2294036.8379780576</v>
+      </c>
+      <c r="X7">
+        <v>46286327.194375373</v>
+      </c>
+      <c r="Y7">
+        <v>336264.36441788985</v>
+      </c>
+      <c r="Z7">
+        <v>6473222.9208265478</v>
+      </c>
+      <c r="AA7">
+        <v>81271631.438536793</v>
+      </c>
+      <c r="AB7">
+        <v>48584558.617720976</v>
+      </c>
+      <c r="AC7">
+        <v>-251686.51610606079</v>
+      </c>
+      <c r="AD7">
+        <v>7965675.0083104493</v>
+      </c>
+      <c r="AE7">
+        <v>7024090.5051082941</v>
+      </c>
+      <c r="AF7">
+        <v>13100728.91200868</v>
+      </c>
+      <c r="AG7">
+        <v>5063268.2234270209</v>
+      </c>
+      <c r="AH7">
+        <v>106933597.08310457</v>
+      </c>
+      <c r="AI7">
+        <v>15353060.711155929</v>
+      </c>
+      <c r="AJ7">
+        <v>23618270.858686872</v>
+      </c>
+      <c r="AK7">
+        <v>1359072.7584565619</v>
+      </c>
+      <c r="AL7">
+        <v>21272286.241695706</v>
+      </c>
+      <c r="AM7">
+        <v>19720360.757326838</v>
+      </c>
+      <c r="AN7">
+        <v>1694787.1288684313</v>
+      </c>
+      <c r="AO7">
+        <v>10112962.434652817</v>
+      </c>
+      <c r="AP7">
+        <v>22898693.827739574</v>
+      </c>
+      <c r="AQ7">
+        <v>29895784.054751128</v>
+      </c>
+      <c r="AR7">
+        <v>-5041050.8470434602</v>
+      </c>
+      <c r="AS7">
+        <v>16593616.638806326</v>
+      </c>
+      <c r="AT7">
+        <v>33755453.046183772</v>
+      </c>
+      <c r="AU7">
+        <v>22673184.480621826</v>
+      </c>
+      <c r="AV7">
+        <v>93730.489014361097</v>
+      </c>
+      <c r="AW7">
+        <v>3222195.622746693</v>
+      </c>
+      <c r="AX7">
+        <v>10515133.319201536</v>
+      </c>
+      <c r="AY7">
+        <v>-8188806.6937705902</v>
+      </c>
+      <c r="AZ7">
+        <v>25818071.113253221</v>
+      </c>
+      <c r="BA7">
+        <v>8373648.8189168433</v>
+      </c>
+      <c r="BB7">
+        <v>47198642.634327292</v>
+      </c>
+      <c r="BC7">
+        <v>3976220.2968137814</v>
+      </c>
+      <c r="BD7">
+        <v>7637749.2086095717</v>
+      </c>
+      <c r="BE7">
+        <v>13619818.688451329</v>
+      </c>
+      <c r="BF7">
+        <v>4500710.7858301727</v>
+      </c>
+      <c r="BG7">
+        <v>15210569.629993754</v>
+      </c>
+      <c r="BH7">
+        <v>46160712.929409645</v>
+      </c>
+      <c r="BI7">
+        <v>16829361.951264199</v>
+      </c>
+      <c r="BJ7">
+        <v>6360065.5376463057</v>
+      </c>
+      <c r="BK7">
+        <v>27722126.752798457</v>
+      </c>
+      <c r="BL7">
+        <v>82497305.877878085</v>
+      </c>
+      <c r="BM7">
+        <v>155007184.92262378</v>
+      </c>
+      <c r="BN7">
+        <v>18568639.366075799</v>
+      </c>
+      <c r="BO7">
+        <v>38587835.092948809</v>
+      </c>
+      <c r="BP7">
+        <v>12218658.591610068</v>
+      </c>
+    </row>
+    <row r="8" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8">
+        <v>8871880.1381225716</v>
+      </c>
+      <c r="D8">
+        <v>45138048.662199169</v>
+      </c>
+      <c r="E8">
+        <v>12363331.739430202</v>
+      </c>
+      <c r="F8">
+        <v>7851908.0841700137</v>
+      </c>
+      <c r="G8">
+        <v>7996180.6817750894</v>
+      </c>
+      <c r="H8">
+        <v>65355948.103019916</v>
+      </c>
+      <c r="I8">
+        <v>14977109.66972906</v>
+      </c>
+      <c r="J8">
+        <v>69147472.86235559</v>
+      </c>
+      <c r="K8">
+        <v>9676829.8270453606</v>
+      </c>
+      <c r="L8">
+        <v>35925576.93377088</v>
+      </c>
+      <c r="M8">
+        <v>11324012.47473694</v>
+      </c>
+      <c r="N8">
+        <v>18577396.89164573</v>
+      </c>
+      <c r="O8">
+        <v>29165583.990245055</v>
+      </c>
+      <c r="P8">
+        <v>14621827.900252853</v>
+      </c>
+      <c r="Q8">
+        <v>3702694.393570479</v>
+      </c>
+      <c r="R8">
+        <v>12031692.87594147</v>
+      </c>
+      <c r="S8">
+        <v>18828714.9456678</v>
+      </c>
+      <c r="T8">
+        <v>7674720.9168675579</v>
+      </c>
+      <c r="U8">
+        <v>43979855.476424649</v>
+      </c>
+      <c r="V8">
+        <v>22117141.820808385</v>
+      </c>
+      <c r="W8">
+        <v>12535084.162078291</v>
+      </c>
+      <c r="X8">
+        <v>29683401.517920773</v>
+      </c>
+      <c r="Y8">
+        <v>1414900.2909470142</v>
+      </c>
+      <c r="Z8">
+        <v>8375522.9104542509</v>
+      </c>
+      <c r="AA8">
+        <v>10773336.694254527</v>
+      </c>
+      <c r="AB8">
+        <v>13465602.205700502</v>
+      </c>
+      <c r="AC8">
+        <v>11713346.704510164</v>
+      </c>
+      <c r="AD8">
+        <v>12387498.214856334</v>
+      </c>
+      <c r="AE8">
+        <v>21231562.432449907</v>
+      </c>
+      <c r="AF8">
+        <v>30010332.262290128</v>
+      </c>
+      <c r="AG8">
+        <v>33816136.000436649</v>
+      </c>
+      <c r="AH8">
+        <v>21413212.828043163</v>
+      </c>
+      <c r="AI8">
+        <v>13982482.204791453</v>
+      </c>
+      <c r="AJ8">
+        <v>34425365.147444658</v>
+      </c>
+      <c r="AK8">
+        <v>8281438.0387904271</v>
+      </c>
+      <c r="AL8">
+        <v>25993825.024637651</v>
+      </c>
+      <c r="AM8">
+        <v>32995531.415888481</v>
+      </c>
+      <c r="AN8">
+        <v>13106960.663701495</v>
+      </c>
+      <c r="AO8">
+        <v>24875452.551099956</v>
+      </c>
+      <c r="AP8">
+        <v>2984564.532710019</v>
+      </c>
+      <c r="AQ8">
+        <v>22181481.203741107</v>
+      </c>
+      <c r="AR8">
+        <v>70536337.173573539</v>
+      </c>
+      <c r="AS8">
+        <v>46392640.212095</v>
+      </c>
+      <c r="AT8">
+        <v>46640971.553289689</v>
+      </c>
+      <c r="AU8">
+        <v>56694346.317172162</v>
+      </c>
+      <c r="AV8">
+        <v>10742660.965076074</v>
+      </c>
+      <c r="AW8">
+        <v>4533498.1470185248</v>
+      </c>
+      <c r="AX8">
+        <v>18415526.777447309</v>
+      </c>
+      <c r="AY8">
+        <v>10791004.098144529</v>
+      </c>
+      <c r="AZ8">
+        <v>26354187.778813612</v>
+      </c>
+      <c r="BA8">
+        <v>22553643.475911289</v>
+      </c>
+      <c r="BB8">
+        <v>19434159.290567372</v>
+      </c>
+      <c r="BC8">
+        <v>9785574.4312297627</v>
+      </c>
+      <c r="BD8">
+        <v>13667940.735201327</v>
+      </c>
+      <c r="BE8">
+        <v>23485797.885791168</v>
+      </c>
+      <c r="BF8">
+        <v>32032729.305865459</v>
+      </c>
+      <c r="BG8">
+        <v>36290170.284067944</v>
+      </c>
+      <c r="BH8">
+        <v>41833246.548166782</v>
+      </c>
+      <c r="BI8">
+        <v>27712050.229939174</v>
+      </c>
+      <c r="BJ8">
+        <v>20718311.396383967</v>
+      </c>
+      <c r="BK8">
+        <v>24407633.169558756</v>
+      </c>
+      <c r="BL8">
+        <v>67581297.238443702</v>
+      </c>
+      <c r="BM8">
+        <v>77763275.58096616</v>
+      </c>
+      <c r="BN8">
+        <v>64720088.419562295</v>
+      </c>
+      <c r="BO8">
+        <v>73855541.00006251</v>
+      </c>
+      <c r="BP8">
+        <v>31161785.738584001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9">
+        <v>11858379.799027113</v>
+      </c>
+      <c r="D9">
+        <v>37565146.800766625</v>
+      </c>
+      <c r="E9">
+        <v>4856973.8948589209</v>
+      </c>
+      <c r="F9">
+        <v>2111921.432174643</v>
+      </c>
+      <c r="G9">
+        <v>5151043.5564121874</v>
+      </c>
+      <c r="H9">
+        <v>153525673.1730535</v>
+      </c>
+      <c r="I9">
+        <v>21240601.500450451</v>
+      </c>
+      <c r="J9">
+        <v>5394371862.3288155</v>
+      </c>
+      <c r="K9">
+        <v>6641024.375397549</v>
+      </c>
+      <c r="L9">
+        <v>23910793.629368596</v>
+      </c>
+      <c r="M9">
+        <v>8946059.7590587009</v>
+      </c>
+      <c r="N9">
+        <v>6473446.5445506759</v>
+      </c>
+      <c r="O9">
+        <v>9104783.011352174</v>
+      </c>
+      <c r="P9">
+        <v>55356832.372478627</v>
+      </c>
+      <c r="Q9">
+        <v>72499017.877583846</v>
+      </c>
+      <c r="R9">
+        <v>531177938.50579143</v>
+      </c>
+      <c r="S9">
+        <v>7656407.4857655792</v>
+      </c>
+      <c r="T9">
+        <v>4642522.7087133462</v>
+      </c>
+      <c r="U9">
+        <v>277785667.48348367</v>
+      </c>
+      <c r="V9">
+        <v>27337073.109406915</v>
+      </c>
+      <c r="W9">
+        <v>46747028.331071489</v>
+      </c>
+      <c r="X9">
+        <v>30473125.639876168</v>
+      </c>
+      <c r="Y9">
+        <v>5503402.3058767896</v>
+      </c>
+      <c r="Z9">
+        <v>7945866.9392261757</v>
+      </c>
+      <c r="AA9">
+        <v>452746046.44947171</v>
+      </c>
+      <c r="AB9">
+        <v>713908614.68089128</v>
+      </c>
+      <c r="AC9">
+        <v>132446942.94500405</v>
+      </c>
+      <c r="AD9">
+        <v>31836496.702737726</v>
+      </c>
+      <c r="AE9">
+        <v>24596802.547829069</v>
+      </c>
+      <c r="AF9">
+        <v>56432525.360473894</v>
+      </c>
+      <c r="AG9">
+        <v>7066541.6415448142</v>
+      </c>
+      <c r="AH9">
+        <v>126215581.5154033</v>
+      </c>
+      <c r="AI9">
+        <v>18639412.306947142</v>
+      </c>
+      <c r="AJ9">
+        <v>62154178.841039024</v>
+      </c>
+      <c r="AK9">
+        <v>1701931.8845594521</v>
+      </c>
+      <c r="AL9">
+        <v>44662318.170798518</v>
+      </c>
+      <c r="AM9">
+        <v>51095177.591312177</v>
+      </c>
+      <c r="AN9">
+        <v>7364706.3594905594</v>
+      </c>
+      <c r="AO9">
+        <v>32016057.950292241</v>
+      </c>
+      <c r="AP9">
+        <v>825689508.52227092</v>
+      </c>
+      <c r="AQ9">
+        <v>23883921.965230908</v>
+      </c>
+      <c r="AR9">
+        <v>137119651.07294545</v>
+      </c>
+      <c r="AS9">
+        <v>63403586.068462178</v>
+      </c>
+      <c r="AT9">
+        <v>22996155.372898918</v>
+      </c>
+      <c r="AU9">
+        <v>20306592.086875375</v>
+      </c>
+      <c r="AV9">
+        <v>1235986.2541022305</v>
+      </c>
+      <c r="AW9">
+        <v>3881334.4111954025</v>
+      </c>
+      <c r="AX9">
+        <v>18104560.740725271</v>
+      </c>
+      <c r="AY9">
+        <v>6217565.1003301367</v>
+      </c>
+      <c r="AZ9">
+        <v>128333796.37207213</v>
+      </c>
+      <c r="BA9">
+        <v>13319715.131807545</v>
+      </c>
+      <c r="BB9">
+        <v>112294392.69659378</v>
+      </c>
+      <c r="BC9">
+        <v>11846182.765112342</v>
+      </c>
+      <c r="BD9">
+        <v>20553151.610407729</v>
+      </c>
+      <c r="BE9">
+        <v>58895914.453191958</v>
+      </c>
+      <c r="BF9">
+        <v>16559966.430310588</v>
+      </c>
+      <c r="BG9">
+        <v>53185262.404111899</v>
+      </c>
+      <c r="BH9">
+        <v>89348321.694379523</v>
+      </c>
+      <c r="BI9">
+        <v>9552225.1047959439</v>
+      </c>
+      <c r="BJ9">
+        <v>40789755.652312398</v>
+      </c>
+      <c r="BK9">
+        <v>46417545.22345186</v>
+      </c>
+      <c r="BL9">
+        <v>151343293.66539356</v>
+      </c>
+      <c r="BM9">
+        <v>297361860.92359787</v>
+      </c>
+      <c r="BN9">
+        <v>22631870.098656334</v>
+      </c>
+      <c r="BO9">
+        <v>64289557.186370559</v>
+      </c>
+      <c r="BP9">
+        <v>9729812.6456108298</v>
+      </c>
+    </row>
+    <row r="10" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10">
+        <v>113685415.27361374</v>
+      </c>
+      <c r="D10">
+        <v>826581516.23730791</v>
+      </c>
+      <c r="E10">
+        <v>147183781.0401305</v>
+      </c>
+      <c r="F10">
+        <v>10609849.114835002</v>
+      </c>
+      <c r="G10">
+        <v>106359253.28903522</v>
+      </c>
+      <c r="H10">
+        <v>3861221761.2824011</v>
+      </c>
+      <c r="I10">
+        <v>867489664.23999</v>
+      </c>
+      <c r="J10">
+        <v>22316402829.895645</v>
+      </c>
+      <c r="K10">
+        <v>2161151437.1927662</v>
+      </c>
+      <c r="L10">
+        <v>654397411.23030674</v>
+      </c>
+      <c r="M10">
+        <v>190151615.11598149</v>
+      </c>
+      <c r="N10">
+        <v>367024164.96328348</v>
+      </c>
+      <c r="O10">
+        <v>418562248.76594502</v>
+      </c>
+      <c r="P10">
+        <v>620487553.51760602</v>
+      </c>
+      <c r="Q10">
+        <v>218616540.96235344</v>
+      </c>
+      <c r="R10">
+        <v>6085542454.1427946</v>
+      </c>
+      <c r="S10">
+        <v>301623964.30974555</v>
+      </c>
+      <c r="T10">
+        <v>107305106.56392169</v>
+      </c>
+      <c r="U10">
+        <v>4060828297.1678638</v>
+      </c>
+      <c r="V10">
+        <v>963759375.15819764</v>
+      </c>
+      <c r="W10">
+        <v>161029085.12938693</v>
+      </c>
+      <c r="X10">
+        <v>852430070.20712984</v>
+      </c>
+      <c r="Y10">
+        <v>137905219.41295943</v>
+      </c>
+      <c r="Z10">
+        <v>248861778.48700485</v>
+      </c>
+      <c r="AA10">
+        <v>8072499710.9324808</v>
+      </c>
+      <c r="AB10">
+        <v>5876981302.215373</v>
+      </c>
+      <c r="AC10">
+        <v>1487760547.0525472</v>
+      </c>
+      <c r="AD10">
+        <v>226087373.52913493</v>
+      </c>
+      <c r="AE10">
+        <v>726737410.15672553</v>
+      </c>
+      <c r="AF10">
+        <v>722557366.98710871</v>
+      </c>
+      <c r="AG10">
+        <v>389014371.596237</v>
+      </c>
+      <c r="AH10">
+        <v>6435986718.4678802</v>
+      </c>
+      <c r="AI10">
+        <v>268789445.7852087</v>
+      </c>
+      <c r="AJ10">
+        <v>1048396420.8048184</v>
+      </c>
+      <c r="AK10">
+        <v>49405803.688497521</v>
+      </c>
+      <c r="AL10">
+        <v>1610981340.1839223</v>
+      </c>
+      <c r="AM10">
+        <v>424820948.5320183</v>
+      </c>
+      <c r="AN10">
+        <v>53930158.81348826</v>
+      </c>
+      <c r="AO10">
+        <v>341337217.6792028</v>
+      </c>
+      <c r="AP10">
+        <v>5164535672.7503881</v>
+      </c>
+      <c r="AQ10">
+        <v>895763425.06682003</v>
+      </c>
+      <c r="AR10">
+        <v>682811077.57802701</v>
+      </c>
+      <c r="AS10">
+        <v>1271539994.8349636</v>
+      </c>
+      <c r="AT10">
+        <v>909680372.86615515</v>
+      </c>
+      <c r="AU10">
+        <v>638593606.71429837</v>
+      </c>
+      <c r="AV10">
+        <v>22908993.678933468</v>
+      </c>
+      <c r="AW10">
+        <v>99700971.394021139</v>
+      </c>
+      <c r="AX10">
+        <v>2047988467.1397614</v>
+      </c>
+      <c r="AY10">
+        <v>291541165.31797051</v>
+      </c>
+      <c r="AZ10">
+        <v>2477438753.6417055</v>
+      </c>
+      <c r="BA10">
+        <v>209774918.28664598</v>
+      </c>
+      <c r="BB10">
+        <v>1633591683.7868729</v>
+      </c>
+      <c r="BC10">
+        <v>568326133.58972657</v>
+      </c>
+      <c r="BD10">
+        <v>-108978132.63665451</v>
+      </c>
+      <c r="BE10">
+        <v>694734041.35768735</v>
+      </c>
+      <c r="BF10">
+        <v>430302130.13433844</v>
+      </c>
+      <c r="BG10">
+        <v>812607313.14017224</v>
+      </c>
+      <c r="BH10">
+        <v>3160573893.752883</v>
+      </c>
+      <c r="BI10">
+        <v>392501641.47209728</v>
+      </c>
+      <c r="BJ10">
+        <v>7934246764.7668276</v>
+      </c>
+      <c r="BK10">
+        <v>1022759140.8154805</v>
+      </c>
+      <c r="BL10">
+        <v>3602551456.6282687</v>
+      </c>
+      <c r="BM10">
+        <v>6172328520.4751139</v>
+      </c>
+      <c r="BN10">
+        <v>496085502.46023285</v>
+      </c>
+      <c r="BO10">
+        <v>1591905266.1216431</v>
+      </c>
+      <c r="BP10">
+        <v>250719575.70337135</v>
+      </c>
+    </row>
+    <row r="11" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11">
+        <v>43044784.993180089</v>
+      </c>
+      <c r="D11">
+        <v>50917994.179771312</v>
+      </c>
+      <c r="E11">
+        <v>39160276.252580777</v>
+      </c>
+      <c r="F11">
+        <v>28958250.094596669</v>
+      </c>
+      <c r="G11">
+        <v>31933061.689027525</v>
+      </c>
+      <c r="H11">
+        <v>159332468.88636753</v>
+      </c>
+      <c r="I11">
+        <v>51851945.690797165</v>
+      </c>
+      <c r="J11">
+        <v>1923868673.7387784</v>
+      </c>
+      <c r="K11">
+        <v>37953736.881179594</v>
+      </c>
+      <c r="L11">
+        <v>114962673.65421957</v>
+      </c>
+      <c r="M11">
+        <v>62051072.753489397</v>
+      </c>
+      <c r="N11">
+        <v>43367887.412846282</v>
+      </c>
+      <c r="O11">
+        <v>34460734.459813125</v>
+      </c>
+      <c r="P11">
+        <v>66376079.785551667</v>
+      </c>
+      <c r="Q11">
+        <v>14625275.861776302</v>
+      </c>
+      <c r="R11">
+        <v>101918655.09380424</v>
+      </c>
+      <c r="S11">
+        <v>114356797.82492791</v>
+      </c>
+      <c r="T11">
+        <v>22720938.199073926</v>
+      </c>
+      <c r="U11">
+        <v>342435750.91005337</v>
+      </c>
+      <c r="V11">
+        <v>148433382.54325998</v>
+      </c>
+      <c r="W11">
+        <v>137091551.4162887</v>
+      </c>
+      <c r="X11">
+        <v>93863290.004885718</v>
+      </c>
+      <c r="Y11">
+        <v>3825899.6722172555</v>
+      </c>
+      <c r="Z11">
+        <v>26676576.355810367</v>
+      </c>
+      <c r="AA11">
+        <v>264845884.85968176</v>
+      </c>
+      <c r="AB11">
+        <v>238455666.89318654</v>
+      </c>
+      <c r="AC11">
+        <v>44548907.201043613</v>
+      </c>
+      <c r="AD11">
+        <v>55497058.543389156</v>
+      </c>
+      <c r="AE11">
+        <v>68912689.804047808</v>
+      </c>
+      <c r="AF11">
+        <v>37952847.815199137</v>
+      </c>
+      <c r="AG11">
+        <v>35788020.936722301</v>
+      </c>
+      <c r="AH11">
+        <v>83856604.933077514</v>
+      </c>
+      <c r="AI11">
+        <v>96236922.91035074</v>
+      </c>
+      <c r="AJ11">
+        <v>62148959.955154069</v>
+      </c>
+      <c r="AK11">
+        <v>8205148.5441889642</v>
+      </c>
+      <c r="AL11">
+        <v>483711063.93405306</v>
+      </c>
+      <c r="AM11">
+        <v>91568933.722952828</v>
+      </c>
+      <c r="AN11">
+        <v>12810137.185447956</v>
+      </c>
+      <c r="AO11">
+        <v>30142801.488003924</v>
+      </c>
+      <c r="AP11">
+        <v>147498180.2058906</v>
+      </c>
+      <c r="AQ11">
+        <v>46869790.115567513</v>
+      </c>
+      <c r="AR11">
+        <v>350163043.25767279</v>
+      </c>
+      <c r="AS11">
+        <v>101743656.0925951</v>
+      </c>
+      <c r="AT11">
+        <v>163671206.45373046</v>
+      </c>
+      <c r="AU11">
+        <v>128625243.08089916</v>
+      </c>
+      <c r="AV11">
+        <v>2196421.8285931055</v>
+      </c>
+      <c r="AW11">
+        <v>8365072.269731381</v>
+      </c>
+      <c r="AX11">
+        <v>138372536.69822088</v>
+      </c>
+      <c r="AY11">
+        <v>130695887.07936318</v>
+      </c>
+      <c r="AZ11">
+        <v>160607938.39595941</v>
+      </c>
+      <c r="BA11">
+        <v>50663149.276873142</v>
+      </c>
+      <c r="BB11">
+        <v>100637334.01914878</v>
+      </c>
+      <c r="BC11">
+        <v>123142587.67611772</v>
+      </c>
+      <c r="BD11">
+        <v>62058705.688714512</v>
+      </c>
+      <c r="BE11">
+        <v>15113367.824520001</v>
+      </c>
+      <c r="BF11">
+        <v>78360113.366860166</v>
+      </c>
+      <c r="BG11">
+        <v>119172067.33848825</v>
+      </c>
+      <c r="BH11">
+        <v>445248952.45902342</v>
+      </c>
+      <c r="BI11">
+        <v>89440569.951614812</v>
+      </c>
+      <c r="BJ11">
+        <v>48231462.021686904</v>
+      </c>
+      <c r="BK11">
+        <v>96899972.670991763</v>
+      </c>
+      <c r="BL11">
+        <v>125554241.50517222</v>
+      </c>
+      <c r="BM11">
+        <v>426964447.60913479</v>
+      </c>
+      <c r="BN11">
+        <v>43322229.527992912</v>
+      </c>
+      <c r="BO11">
+        <v>221371228.78508192</v>
+      </c>
+      <c r="BP11">
+        <v>29951451.049896631</v>
+      </c>
+    </row>
+    <row r="12" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12">
+        <v>349825222.68432504</v>
+      </c>
+      <c r="D12">
+        <v>1211805655.0013402</v>
+      </c>
+      <c r="E12">
+        <v>342529489.39554763</v>
+      </c>
+      <c r="F12">
+        <v>123806128.85217679</v>
+      </c>
+      <c r="G12">
+        <v>187819656.56190279</v>
+      </c>
+      <c r="H12">
+        <v>1449094992.9749758</v>
+      </c>
+      <c r="I12">
+        <v>729995460.80383694</v>
+      </c>
+      <c r="J12">
+        <v>34821044879.517792</v>
+      </c>
+      <c r="K12">
+        <v>265546718.63526762</v>
+      </c>
+      <c r="L12">
+        <v>1142826744.011512</v>
+      </c>
+      <c r="M12">
+        <v>392005864.37384599</v>
+      </c>
+      <c r="N12">
+        <v>536545099.1389004</v>
+      </c>
+      <c r="O12">
+        <v>871482134.17178154</v>
+      </c>
+      <c r="P12">
+        <v>917486577.43799484</v>
+      </c>
+      <c r="Q12">
+        <v>166170876.34673676</v>
+      </c>
+      <c r="R12">
+        <v>1210031821.8047814</v>
+      </c>
+      <c r="S12">
+        <v>650903730.41295028</v>
+      </c>
+      <c r="T12">
+        <v>322437257.50903893</v>
+      </c>
+      <c r="U12">
+        <v>3539206819.4183145</v>
+      </c>
+      <c r="V12">
+        <v>808939987.51501632</v>
+      </c>
+      <c r="W12">
+        <v>2526944439.4058924</v>
+      </c>
+      <c r="X12">
+        <v>2197702803.9856505</v>
+      </c>
+      <c r="Y12">
+        <v>46491571.645314373</v>
+      </c>
+      <c r="Z12">
+        <v>316837774.27343297</v>
+      </c>
+      <c r="AA12">
+        <v>2966748092.1845608</v>
+      </c>
+      <c r="AB12">
+        <v>1866560636.2387493</v>
+      </c>
+      <c r="AC12">
+        <v>289384744.68696845</v>
+      </c>
+      <c r="AD12">
+        <v>582509689.01307631</v>
+      </c>
+      <c r="AE12">
+        <v>808450262.08812714</v>
+      </c>
+      <c r="AF12">
+        <v>719612599.24460649</v>
+      </c>
+      <c r="AG12">
+        <v>823328525.5459255</v>
+      </c>
+      <c r="AH12">
+        <v>3692292640.9022059</v>
+      </c>
+      <c r="AI12">
+        <v>614927248.74317181</v>
+      </c>
+      <c r="AJ12">
+        <v>1108534762.949235</v>
+      </c>
+      <c r="AK12">
+        <v>194019569.92757672</v>
+      </c>
+      <c r="AL12">
+        <v>2709757813.785274</v>
+      </c>
+      <c r="AM12">
+        <v>919192085.06739247</v>
+      </c>
+      <c r="AN12">
+        <v>230434340.84089205</v>
+      </c>
+      <c r="AO12">
+        <v>494951715.82145423</v>
+      </c>
+      <c r="AP12">
+        <v>1053522619.1835042</v>
+      </c>
+      <c r="AQ12">
+        <v>823726653.80827081</v>
+      </c>
+      <c r="AR12">
+        <v>885939431.44755816</v>
+      </c>
+      <c r="AS12">
+        <v>1119598995.5430624</v>
+      </c>
+      <c r="AT12">
+        <v>1600079592.4414933</v>
+      </c>
+      <c r="AU12">
+        <v>1217526636.1619999</v>
+      </c>
+      <c r="AV12">
+        <v>132133836.92708641</v>
+      </c>
+      <c r="AW12">
+        <v>174701582.3901813</v>
+      </c>
+      <c r="AX12">
+        <v>786677210.62706888</v>
+      </c>
+      <c r="AY12">
+        <v>425452394.09323657</v>
+      </c>
+      <c r="AZ12">
+        <v>2303979044.695251</v>
+      </c>
+      <c r="BA12">
+        <v>576529440.93334103</v>
+      </c>
+      <c r="BB12">
+        <v>2457382722.6636028</v>
+      </c>
+      <c r="BC12">
+        <v>702693066.47125459</v>
+      </c>
+      <c r="BD12">
+        <v>499898834.66249382</v>
+      </c>
+      <c r="BE12">
+        <v>677905429.05937612</v>
+      </c>
+      <c r="BF12">
+        <v>719673154.99681485</v>
+      </c>
+      <c r="BG12">
+        <v>1684628979.8663764</v>
+      </c>
+      <c r="BH12">
+        <v>2251872163.9236827</v>
+      </c>
+      <c r="BI12">
+        <v>880832411.83053112</v>
+      </c>
+      <c r="BJ12">
+        <v>593452432.04593349</v>
+      </c>
+      <c r="BK12">
+        <v>1083356017.4590206</v>
+      </c>
+      <c r="BL12">
+        <v>3057903585.6772418</v>
+      </c>
+      <c r="BM12">
+        <v>5149648795.6344976</v>
+      </c>
+      <c r="BN12">
+        <v>734984068.42425299</v>
+      </c>
+      <c r="BO12">
+        <v>2671234276.242569</v>
+      </c>
+      <c r="BP12">
+        <v>693889107.71635759</v>
+      </c>
+    </row>
+    <row r="13" spans="1:68" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13">
+        <v>4299131.5157287708</v>
+      </c>
+      <c r="D13">
+        <v>30747615.996222232</v>
+      </c>
+      <c r="E13">
+        <v>213596.81363646564</v>
+      </c>
+      <c r="F13">
+        <v>-1692858.009666027</v>
+      </c>
+      <c r="G13">
+        <v>2425720.9851564309</v>
+      </c>
+      <c r="H13">
+        <v>19141228.086659651</v>
+      </c>
+      <c r="I13">
+        <v>14123018.756889632</v>
+      </c>
+      <c r="J13">
+        <v>656647835.31169951</v>
+      </c>
+      <c r="K13">
+        <v>1295255.1137813495</v>
+      </c>
+      <c r="L13">
+        <v>20705601.693422098</v>
+      </c>
+      <c r="M13">
+        <v>-786967.20729905099</v>
+      </c>
+      <c r="N13">
+        <v>8920285.6511230357</v>
+      </c>
+      <c r="O13">
+        <v>13076225.53963518</v>
+      </c>
+      <c r="P13">
+        <v>11271388.729813512</v>
+      </c>
+      <c r="Q13">
+        <v>93134.234469822273</v>
+      </c>
+      <c r="R13">
+        <v>31901258.9106405</v>
+      </c>
+      <c r="S13">
+        <v>1420426.2766954436</v>
+      </c>
+      <c r="T13">
+        <v>929887.12228463183</v>
+      </c>
+      <c r="U13">
+        <v>74872371.59119828</v>
+      </c>
+      <c r="V13">
+        <v>16213669.323804984</v>
+      </c>
+      <c r="W13">
+        <v>-5310695.2799192034</v>
+      </c>
+      <c r="X13">
+        <v>48772140.790148698</v>
+      </c>
+      <c r="Y13">
+        <v>341583.53937085508</v>
+      </c>
+      <c r="Z13">
+        <v>6854174.4522073073</v>
+      </c>
+      <c r="AA13">
+        <v>88852452.640587509</v>
+      </c>
+      <c r="AB13">
+        <v>50820228.547937289</v>
+      </c>
+      <c r="AC13">
+        <v>411850.66271900857</v>
+      </c>
+      <c r="AD13">
+        <v>7946595.5472126994</v>
+      </c>
+      <c r="AE13">
+        <v>7195839.4265498137</v>
+      </c>
+      <c r="AF13">
+        <v>15544999.586134253</v>
+      </c>
+      <c r="AG13">
+        <v>5233524.3186592162</v>
+      </c>
+      <c r="AH13">
+        <v>115248273.56972672</v>
+      </c>
+      <c r="AI13">
+        <v>16426512.076977056</v>
+      </c>
+      <c r="AJ13">
+        <v>25769781.714800622</v>
+      </c>
+      <c r="AK13">
+        <v>1451496.3872577867</v>
+      </c>
+      <c r="AL13">
+        <v>23043009.291781362</v>
+      </c>
+      <c r="AM13">
+        <v>21060344.337235253</v>
+      </c>
+      <c r="AN13">
+        <v>1804482.0886657408</v>
+      </c>
+      <c r="AO13">
+        <v>10447024.256818525</v>
+      </c>
+      <c r="AP13">
+        <v>23370492.502676226</v>
+      </c>
+      <c r="AQ13">
+        <v>31045621.903010786</v>
+      </c>
+      <c r="AR13">
+        <v>-2353110.4507416887</v>
+      </c>
+      <c r="AS13">
+        <v>18217456.799178809</v>
+      </c>
+      <c r="AT13">
+        <v>34352508.082807384</v>
+      </c>
+      <c r="AU13">
+        <v>24277777.519660808</v>
+      </c>
+      <c r="AV13">
+        <v>111589.62311044781</v>
+      </c>
+      <c r="AW13">
+        <v>3497875.6530276891</v>
+      </c>
+      <c r="AX13">
+        <v>11150857.409950208</v>
+      </c>
+      <c r="AY13">
+        <v>-7942241.5819720542</v>
+      </c>
+      <c r="AZ13">
+        <v>28815753.94079366</v>
+      </c>
+      <c r="BA13">
+        <v>9261695.1317960788</v>
+      </c>
+      <c r="BB13">
+        <v>49836751.602820404</v>
+      </c>
+      <c r="BC13">
+        <v>4903061.6827258896</v>
+      </c>
+      <c r="BD13">
+        <v>7997341.9208793258</v>
+      </c>
+      <c r="BE13">
+        <v>14330417.924370529</v>
+      </c>
+      <c r="BF13">
+        <v>5268959.0015383437</v>
+      </c>
+      <c r="BG13">
+        <v>15384634.247238403</v>
+      </c>
+      <c r="BH13">
+        <v>52947026.695897475</v>
+      </c>
+      <c r="BI13">
+        <v>17826814.677253377</v>
+      </c>
+      <c r="BJ13">
+        <v>6538385.1321597537</v>
+      </c>
+      <c r="BK13">
+        <v>28876714.244455133</v>
+      </c>
+      <c r="BL13">
+        <v>84534276.393381253</v>
+      </c>
+      <c r="BM13">
+        <v>155007184.92262378</v>
+      </c>
+      <c r="BN13">
+        <v>19605062.2502869</v>
+      </c>
+      <c r="BO13">
+        <v>42525712.72563526</v>
+      </c>
+      <c r="BP13">
+        <v>12882413.215495996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>